<commit_message>
Mi descripción de cambios
</commit_message>
<xml_diff>
--- a/Asegurados_SIS/Data/Asegurados_Por_Establecimiento.xlsx
+++ b/Asegurados_SIS/Data/Asegurados_Por_Establecimiento.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\proyectos_python\DashboardExcel\Asegurados_SIS\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FCFC584E-2297-4495-ABA8-A2327D96C2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C374B04-25C9-4398-8262-C173B328CD58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-48" yWindow="-48" windowWidth="23136" windowHeight="12336" xr2:uid="{7419DD17-BEFA-4D2D-9BB8-937CAA02C6C8}"/>
+    <workbookView xWindow="-48" yWindow="-48" windowWidth="23136" windowHeight="12336" xr2:uid="{F0D998CC-A976-4A0A-851B-F3CAA0C961F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -160,6 +160,15 @@
     <t>00004993</t>
   </si>
   <si>
+    <t>SILLANGATE</t>
+  </si>
+  <si>
+    <t>C.S. SILLANGATE</t>
+  </si>
+  <si>
+    <t>00004968</t>
+  </si>
+  <si>
     <t>CHOROS</t>
   </si>
   <si>
@@ -169,15 +178,6 @@
     <t>00004971</t>
   </si>
   <si>
-    <t>SILLANGATE</t>
-  </si>
-  <si>
-    <t>C.S. SILLANGATE</t>
-  </si>
-  <si>
-    <t>00004968</t>
-  </si>
-  <si>
     <t>SAN JUAN</t>
   </si>
   <si>
@@ -265,6 +265,12 @@
     <t>SUMIDERO</t>
   </si>
   <si>
+    <t>00004982</t>
+  </si>
+  <si>
+    <t>SALABAMBA</t>
+  </si>
+  <si>
     <t>00004989</t>
   </si>
   <si>
@@ -280,12 +286,6 @@
     <t>LA SACILIA</t>
   </si>
   <si>
-    <t>00004982</t>
-  </si>
-  <si>
-    <t>SALABAMBA</t>
-  </si>
-  <si>
     <t>CUJILLO</t>
   </si>
   <si>
@@ -313,18 +313,18 @@
     <t>SAN JOSE DE LIRIO</t>
   </si>
   <si>
+    <t>00004991</t>
+  </si>
+  <si>
+    <t>LANCHE</t>
+  </si>
+  <si>
     <t>00004972</t>
   </si>
   <si>
     <t>MESARRUME</t>
   </si>
   <si>
-    <t>00004991</t>
-  </si>
-  <si>
-    <t>LANCHE</t>
-  </si>
-  <si>
     <t>00007698</t>
   </si>
   <si>
@@ -349,36 +349,42 @@
     <t>MINAS</t>
   </si>
   <si>
+    <t>00004998</t>
+  </si>
+  <si>
+    <t>EL CARDON</t>
+  </si>
+  <si>
+    <t>00004975</t>
+  </si>
+  <si>
+    <t>YUNCHACO</t>
+  </si>
+  <si>
+    <t>00004983</t>
+  </si>
+  <si>
+    <t>CRUZ ROJA</t>
+  </si>
+  <si>
     <t>00004988</t>
   </si>
   <si>
     <t>LA COLCA</t>
   </si>
   <si>
-    <t>00004983</t>
-  </si>
-  <si>
-    <t>CRUZ ROJA</t>
-  </si>
-  <si>
-    <t>00004998</t>
-  </si>
-  <si>
-    <t>EL CARDON</t>
-  </si>
-  <si>
-    <t>00004975</t>
-  </si>
-  <si>
-    <t>YUNCHACO</t>
-  </si>
-  <si>
     <t>00005011</t>
   </si>
   <si>
     <t>PARIC</t>
   </si>
   <si>
+    <t>00004963</t>
+  </si>
+  <si>
+    <t>SANTA CLARA</t>
+  </si>
+  <si>
     <t>00004969</t>
   </si>
   <si>
@@ -391,12 +397,6 @@
     <t>CULLANMAYO</t>
   </si>
   <si>
-    <t>00004963</t>
-  </si>
-  <si>
-    <t>SANTA CLARA</t>
-  </si>
-  <si>
     <t>00006937</t>
   </si>
   <si>
@@ -406,22 +406,34 @@
     <t>CHUGUR</t>
   </si>
   <si>
+    <t>00006938</t>
+  </si>
+  <si>
+    <t>CACHACARA</t>
+  </si>
+  <si>
+    <t>00007752</t>
+  </si>
+  <si>
+    <t>SANTA CLARA DE CAMSE</t>
+  </si>
+  <si>
+    <t>00004967</t>
+  </si>
+  <si>
+    <t>SECTOR EL CAMPO</t>
+  </si>
+  <si>
     <t>00005024</t>
   </si>
   <si>
     <t>LANCHEPATA</t>
   </si>
   <si>
-    <t>00006938</t>
-  </si>
-  <si>
-    <t>CACHACARA</t>
-  </si>
-  <si>
-    <t>00004967</t>
-  </si>
-  <si>
-    <t>SECTOR EL CAMPO</t>
+    <t>00005035</t>
+  </si>
+  <si>
+    <t>LA FLOR</t>
   </si>
   <si>
     <t>00005031</t>
@@ -430,18 +442,6 @@
     <t>SANTA CRUZ DE LA SUCCHA</t>
   </si>
   <si>
-    <t>00007752</t>
-  </si>
-  <si>
-    <t>SANTA CLARA DE CAMSE</t>
-  </si>
-  <si>
-    <t>00005035</t>
-  </si>
-  <si>
-    <t>LA FLOR</t>
-  </si>
-  <si>
     <t>00005026</t>
   </si>
   <si>
@@ -454,52 +454,58 @@
     <t>CONDORHUASI</t>
   </si>
   <si>
+    <t>00004994</t>
+  </si>
+  <si>
+    <t>PAYAC</t>
+  </si>
+  <si>
     <t>00005009</t>
   </si>
   <si>
     <t>QUIPAYUC</t>
   </si>
   <si>
-    <t>00004994</t>
-  </si>
-  <si>
-    <t>PAYAC</t>
-  </si>
-  <si>
     <t>00007746</t>
   </si>
   <si>
     <t>LAGUNAS</t>
   </si>
   <si>
+    <t>00005037</t>
+  </si>
+  <si>
+    <t>CHISIGLE</t>
+  </si>
+  <si>
+    <t>00007747</t>
+  </si>
+  <si>
+    <t>PAJURILLO</t>
+  </si>
+  <si>
+    <t>00004979</t>
+  </si>
+  <si>
+    <t>CAMPO FLORIDO</t>
+  </si>
+  <si>
+    <t>00004990</t>
+  </si>
+  <si>
+    <t>YATUN</t>
+  </si>
+  <si>
     <t>00006850</t>
   </si>
   <si>
     <t>CONDAY</t>
   </si>
   <si>
-    <t>00005037</t>
-  </si>
-  <si>
-    <t>CHISIGLE</t>
-  </si>
-  <si>
-    <t>00007747</t>
-  </si>
-  <si>
-    <t>PAJURILLO</t>
-  </si>
-  <si>
-    <t>00004979</t>
-  </si>
-  <si>
-    <t>CAMPO FLORIDO</t>
-  </si>
-  <si>
-    <t>00004990</t>
-  </si>
-  <si>
-    <t>YATUN</t>
+    <t>00007749</t>
+  </si>
+  <si>
+    <t>CHURUMAYO</t>
   </si>
   <si>
     <t>00005021</t>
@@ -508,42 +514,36 @@
     <t>VIZA</t>
   </si>
   <si>
+    <t>00011068</t>
+  </si>
+  <si>
+    <t>PUCALA</t>
+  </si>
+  <si>
+    <t>00005036</t>
+  </si>
+  <si>
+    <t>QUILLUGAY</t>
+  </si>
+  <si>
+    <t>00004985</t>
+  </si>
+  <si>
+    <t>REJOPAMPA</t>
+  </si>
+  <si>
+    <t>00006864</t>
+  </si>
+  <si>
+    <t>NARANJOYACU</t>
+  </si>
+  <si>
     <t>00005023</t>
   </si>
   <si>
     <t>TAMBILLO</t>
   </si>
   <si>
-    <t>00007749</t>
-  </si>
-  <si>
-    <t>CHURUMAYO</t>
-  </si>
-  <si>
-    <t>00005036</t>
-  </si>
-  <si>
-    <t>QUILLUGAY</t>
-  </si>
-  <si>
-    <t>00004985</t>
-  </si>
-  <si>
-    <t>REJOPAMPA</t>
-  </si>
-  <si>
-    <t>00006864</t>
-  </si>
-  <si>
-    <t>NARANJOYACU</t>
-  </si>
-  <si>
-    <t>00011068</t>
-  </si>
-  <si>
-    <t>PUCALA</t>
-  </si>
-  <si>
     <t>00005028</t>
   </si>
   <si>
@@ -574,18 +574,18 @@
     <t>ADCUÑAC</t>
   </si>
   <si>
+    <t>00005022</t>
+  </si>
+  <si>
+    <t>EL ARENAL DE SANTO TOMAS</t>
+  </si>
+  <si>
     <t>00004965</t>
   </si>
   <si>
     <t>QUEROMARCA</t>
   </si>
   <si>
-    <t>00005022</t>
-  </si>
-  <si>
-    <t>EL ARENAL DE SANTO TOMAS</t>
-  </si>
-  <si>
     <t>00006870</t>
   </si>
   <si>
@@ -604,6 +604,12 @@
     <t>CUNUAT</t>
   </si>
   <si>
+    <t>00005041</t>
+  </si>
+  <si>
+    <t>MOCHADIN</t>
+  </si>
+  <si>
     <t>00006943</t>
   </si>
   <si>
@@ -616,12 +622,6 @@
     <t>LAS DELICIAS</t>
   </si>
   <si>
-    <t>00005041</t>
-  </si>
-  <si>
-    <t>MOCHADIN</t>
-  </si>
-  <si>
     <t>00007701</t>
   </si>
   <si>
@@ -640,46 +640,64 @@
     <t>AULLAN</t>
   </si>
   <si>
+    <t>00005039</t>
+  </si>
+  <si>
+    <t>SANTO DOMINGO DE LA LUCMA</t>
+  </si>
+  <si>
     <t>00007109</t>
   </si>
   <si>
     <t>CHIPULUC</t>
   </si>
   <si>
-    <t>00005039</t>
-  </si>
-  <si>
-    <t>SANTO DOMINGO DE LA LUCMA</t>
-  </si>
-  <si>
     <t>00005042</t>
   </si>
   <si>
     <t>SAN ANTONIO</t>
   </si>
   <si>
+    <t>00004997</t>
+  </si>
+  <si>
+    <t>TRIGOPAMPA</t>
+  </si>
+  <si>
+    <t>00005025</t>
+  </si>
+  <si>
+    <t>SAN LUIS</t>
+  </si>
+  <si>
     <t>00007431</t>
   </si>
   <si>
     <t>CONGA DE ALLANGA</t>
   </si>
   <si>
-    <t>00005025</t>
-  </si>
-  <si>
-    <t>SAN LUIS</t>
-  </si>
-  <si>
     <t>00006828</t>
   </si>
   <si>
     <t>SANTA ROSA DE CALLAYUC</t>
   </si>
   <si>
-    <t>00004997</t>
-  </si>
-  <si>
-    <t>TRIGOPAMPA</t>
+    <t>00007097</t>
+  </si>
+  <si>
+    <t>AÑALCATE</t>
+  </si>
+  <si>
+    <t>00004986</t>
+  </si>
+  <si>
+    <t>EL ARENAL DE CUTERVO</t>
+  </si>
+  <si>
+    <t>00007101</t>
+  </si>
+  <si>
+    <t>EL GUAYO</t>
   </si>
   <si>
     <t>00005016</t>
@@ -688,10 +706,10 @@
     <t>PANDALLE</t>
   </si>
   <si>
-    <t>00007097</t>
-  </si>
-  <si>
-    <t>AÑALCATE</t>
+    <t>00004996</t>
+  </si>
+  <si>
+    <t>RAMBRAN</t>
   </si>
   <si>
     <t>00005032</t>
@@ -706,28 +724,16 @@
     <t>RAYME</t>
   </si>
   <si>
-    <t>00007101</t>
-  </si>
-  <si>
-    <t>EL GUAYO</t>
-  </si>
-  <si>
     <t>00005017</t>
   </si>
   <si>
     <t>PERLAMAYO</t>
   </si>
   <si>
-    <t>00004996</t>
-  </si>
-  <si>
-    <t>RAMBRAN</t>
-  </si>
-  <si>
-    <t>00004986</t>
-  </si>
-  <si>
-    <t>EL ARENAL DE CUTERVO</t>
+    <t>00006860</t>
+  </si>
+  <si>
+    <t>TECHIN</t>
   </si>
   <si>
     <t>00007366</t>
@@ -736,10 +742,10 @@
     <t>EL CORRAL</t>
   </si>
   <si>
-    <t>00006860</t>
-  </si>
-  <si>
-    <t>TECHIN</t>
+    <t>00007753</t>
+  </si>
+  <si>
+    <t>BARBASCO</t>
   </si>
   <si>
     <t>00006861</t>
@@ -754,12 +760,6 @@
     <t>LA SUCCHA</t>
   </si>
   <si>
-    <t>00007753</t>
-  </si>
-  <si>
-    <t>BARBASCO</t>
-  </si>
-  <si>
     <t>00011067</t>
   </si>
   <si>
@@ -772,75 +772,81 @@
     <t>SAN CRISTOBAL DE NUDILLO</t>
   </si>
   <si>
+    <t>00006851</t>
+  </si>
+  <si>
+    <t>HUICHUD</t>
+  </si>
+  <si>
+    <t>00006854</t>
+  </si>
+  <si>
+    <t>CARAMARCA CHICA</t>
+  </si>
+  <si>
+    <t>00004962</t>
+  </si>
+  <si>
+    <t>HUABAL</t>
+  </si>
+  <si>
+    <t>00004995</t>
+  </si>
+  <si>
+    <t>PALMAS DE HUICHUD</t>
+  </si>
+  <si>
     <t>00006947</t>
   </si>
   <si>
     <t>LAGUNA</t>
   </si>
   <si>
-    <t>00006854</t>
-  </si>
-  <si>
-    <t>CARAMARCA CHICA</t>
-  </si>
-  <si>
-    <t>00006851</t>
-  </si>
-  <si>
-    <t>HUICHUD</t>
-  </si>
-  <si>
-    <t>00004995</t>
-  </si>
-  <si>
-    <t>PALMAS DE HUICHUD</t>
-  </si>
-  <si>
-    <t>00004962</t>
-  </si>
-  <si>
-    <t>HUABAL</t>
-  </si>
-  <si>
     <t>00008922</t>
   </si>
   <si>
     <t>LA CASCARILLA</t>
   </si>
   <si>
+    <t>00006868</t>
+  </si>
+  <si>
+    <t>ILLUGAN</t>
+  </si>
+  <si>
+    <t>00006859</t>
+  </si>
+  <si>
+    <t>MOSHOQUEQUE</t>
+  </si>
+  <si>
     <t>00006853</t>
   </si>
   <si>
     <t>SAIREPAMPA</t>
   </si>
   <si>
-    <t>00006868</t>
-  </si>
-  <si>
-    <t>ILLUGAN</t>
-  </si>
-  <si>
-    <t>00006859</t>
-  </si>
-  <si>
-    <t>MOSHOQUEQUE</t>
+    <t>00004999</t>
+  </si>
+  <si>
+    <t>LAS PALMAS DE TINTAYOC</t>
   </si>
   <si>
     <t>00007180</t>
   </si>
   <si>
-    <t>00004999</t>
-  </si>
-  <si>
-    <t>LAS PALMAS DE TINTAYOC</t>
-  </si>
-  <si>
     <t>00007098</t>
   </si>
   <si>
     <t>YACANCATE</t>
   </si>
   <si>
+    <t>00006940</t>
+  </si>
+  <si>
+    <t>PAJONAL</t>
+  </si>
+  <si>
     <t>00006862</t>
   </si>
   <si>
@@ -853,18 +859,18 @@
     <t>NARANJOS</t>
   </si>
   <si>
-    <t>00006940</t>
-  </si>
-  <si>
-    <t>PAJONAL</t>
-  </si>
-  <si>
     <t>00005030</t>
   </si>
   <si>
     <t>MUSUNGATE</t>
   </si>
   <si>
+    <t>00006787</t>
+  </si>
+  <si>
+    <t>SANTA ROSA DE TAPO</t>
+  </si>
+  <si>
     <t>00006944</t>
   </si>
   <si>
@@ -883,12 +889,6 @@
     <t>MARAYBAMBA ALTO</t>
   </si>
   <si>
-    <t>00006787</t>
-  </si>
-  <si>
-    <t>SANTA ROSA DE TAPO</t>
-  </si>
-  <si>
     <t>00006942</t>
   </si>
   <si>
@@ -907,16 +907,34 @@
     <t>LA CONGONA</t>
   </si>
   <si>
+    <t>00007367</t>
+  </si>
+  <si>
+    <t>CONGA</t>
+  </si>
+  <si>
     <t>00004970</t>
   </si>
   <si>
     <t>SANTOS</t>
   </si>
   <si>
-    <t>00007367</t>
-  </si>
-  <si>
-    <t>CONGA</t>
+    <t>00006936</t>
+  </si>
+  <si>
+    <t>CORRALES</t>
+  </si>
+  <si>
+    <t>00007369</t>
+  </si>
+  <si>
+    <t>CHONTAS</t>
+  </si>
+  <si>
+    <t>00007370</t>
+  </si>
+  <si>
+    <t>CEDROPAMPA</t>
   </si>
   <si>
     <t>00011258</t>
@@ -925,28 +943,16 @@
     <t>RINCONADA MIRAFLORES</t>
   </si>
   <si>
-    <t>00007369</t>
-  </si>
-  <si>
-    <t>CHONTAS</t>
-  </si>
-  <si>
-    <t>00007370</t>
-  </si>
-  <si>
-    <t>CEDROPAMPA</t>
-  </si>
-  <si>
     <t>00011261</t>
   </si>
   <si>
     <t>GRAMALOTILLO</t>
   </si>
   <si>
-    <t>00006936</t>
-  </si>
-  <si>
-    <t>CORRALES</t>
+    <t>00008925</t>
+  </si>
+  <si>
+    <t>LA LLICA</t>
   </si>
   <si>
     <t>00007048</t>
@@ -961,64 +967,70 @@
     <t>FILADELFIA</t>
   </si>
   <si>
-    <t>00008925</t>
-  </si>
-  <si>
-    <t>LA LLICA</t>
-  </si>
-  <si>
     <t>00005043</t>
   </si>
   <si>
     <t>LAGUNA SHITA</t>
   </si>
   <si>
+    <t>00011066</t>
+  </si>
+  <si>
+    <t>VISTA ALEGRE DE LA SOLA</t>
+  </si>
+  <si>
+    <t>00005000</t>
+  </si>
+  <si>
+    <t>MUNUNO</t>
+  </si>
+  <si>
+    <t>00011260</t>
+  </si>
+  <si>
+    <t>LA VIÑA</t>
+  </si>
+  <si>
+    <t>00011262</t>
+  </si>
+  <si>
+    <t>EL PUQUIO</t>
+  </si>
+  <si>
+    <t>00006960</t>
+  </si>
+  <si>
+    <t>PAN DE AZUCAR</t>
+  </si>
+  <si>
+    <t>00007047</t>
+  </si>
+  <si>
+    <t>ANDAMARCA</t>
+  </si>
+  <si>
     <t>00006835</t>
   </si>
   <si>
     <t>CHURAS</t>
   </si>
   <si>
-    <t>00011066</t>
-  </si>
-  <si>
-    <t>VISTA ALEGRE DE LA SOLA</t>
-  </si>
-  <si>
-    <t>00006960</t>
-  </si>
-  <si>
-    <t>PAN DE AZUCAR</t>
-  </si>
-  <si>
     <t>00007100</t>
   </si>
   <si>
     <t>SAN JUAN DE CHORRILLOS</t>
   </si>
   <si>
-    <t>00005000</t>
-  </si>
-  <si>
-    <t>MUNUNO</t>
-  </si>
-  <si>
-    <t>00011262</t>
-  </si>
-  <si>
-    <t>EL PUQUIO</t>
-  </si>
-  <si>
-    <t>00007047</t>
-  </si>
-  <si>
-    <t>ANDAMARCA</t>
-  </si>
-  <si>
-    <t>00011260</t>
-  </si>
-  <si>
-    <t>LA VIÑA</t>
+    <t>00004980</t>
+  </si>
+  <si>
+    <t>SAN JUAN DE LIMON</t>
+  </si>
+  <si>
+    <t>00007750</t>
+  </si>
+  <si>
+    <t>TAYALES</t>
   </si>
   <si>
     <t>00006829</t>
@@ -1027,10 +1039,10 @@
     <t>PUQUIO</t>
   </si>
   <si>
-    <t>00007750</t>
-  </si>
-  <si>
-    <t>TAYALES</t>
+    <t>00006833</t>
+  </si>
+  <si>
+    <t>LA JAYUA</t>
   </si>
   <si>
     <t>00006958</t>
@@ -1039,18 +1051,6 @@
     <t>PLAYA HERMOZA</t>
   </si>
   <si>
-    <t>00004980</t>
-  </si>
-  <si>
-    <t>SAN JUAN DE LIMON</t>
-  </si>
-  <si>
-    <t>00006833</t>
-  </si>
-  <si>
-    <t>LA JAYUA</t>
-  </si>
-  <si>
     <t>00006831</t>
   </si>
   <si>
@@ -1060,13 +1060,19 @@
     <t>CUÑANQUE</t>
   </si>
   <si>
+    <t>00005033</t>
+  </si>
+  <si>
+    <t>EL PORVENIR</t>
+  </si>
+  <si>
     <t>00006836</t>
   </si>
   <si>
-    <t>00005033</t>
-  </si>
-  <si>
-    <t>EL PORVENIR</t>
+    <t>00006852</t>
+  </si>
+  <si>
+    <t>LLIPA</t>
   </si>
   <si>
     <t>00008923</t>
@@ -1078,19 +1084,19 @@
     <t>00011061</t>
   </si>
   <si>
-    <t>00006852</t>
-  </si>
-  <si>
-    <t>LLIPA</t>
+    <t>00007179</t>
+  </si>
+  <si>
+    <t>CHACRERIAS</t>
   </si>
   <si>
     <t>00007103</t>
   </si>
   <si>
-    <t>00007179</t>
-  </si>
-  <si>
-    <t>CHACRERIAS</t>
+    <t>00006788</t>
+  </si>
+  <si>
+    <t>YANGACHIS</t>
   </si>
   <si>
     <t>00007049</t>
@@ -1099,34 +1105,28 @@
     <t>SURO CHICO</t>
   </si>
   <si>
+    <t>00007368</t>
+  </si>
+  <si>
+    <t>CUCHEA</t>
+  </si>
+  <si>
+    <t>00011064</t>
+  </si>
+  <si>
+    <t>SAN LORENZO</t>
+  </si>
+  <si>
     <t>00006948</t>
   </si>
   <si>
     <t>SANTA ELENA</t>
   </si>
   <si>
-    <t>00007368</t>
-  </si>
-  <si>
-    <t>CUCHEA</t>
-  </si>
-  <si>
-    <t>00011064</t>
-  </si>
-  <si>
-    <t>SAN LORENZO</t>
-  </si>
-  <si>
     <t>00011065</t>
   </si>
   <si>
     <t>PALMA CENTRAL</t>
-  </si>
-  <si>
-    <t>00006788</t>
-  </si>
-  <si>
-    <t>YANGACHIS</t>
   </si>
   <si>
     <t>00004978</t>
@@ -2074,7 +2074,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{994FC810-A3BB-4608-888B-FA77951767C3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1571260C-566B-4744-ABBE-74B1A8E7A7EA}">
   <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2135,7 +2135,7 @@
         <v>3</v>
       </c>
       <c r="H2" s="1">
-        <v>17864</v>
+        <v>17914</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -2158,7 +2158,7 @@
         <v>4</v>
       </c>
       <c r="H3" s="1">
-        <v>7545</v>
+        <v>7373</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -2181,7 +2181,7 @@
         <v>7</v>
       </c>
       <c r="H4" s="1">
-        <v>4743</v>
+        <v>4712</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -2204,7 +2204,7 @@
         <v>10</v>
       </c>
       <c r="H5" s="1">
-        <v>3962</v>
+        <v>3957</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -2227,7 +2227,7 @@
         <v>13</v>
       </c>
       <c r="H6" s="1">
-        <v>3333</v>
+        <v>3268</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -2250,7 +2250,7 @@
         <v>16</v>
       </c>
       <c r="H7" s="1">
-        <v>2912</v>
+        <v>2918</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -2273,7 +2273,7 @@
         <v>19</v>
       </c>
       <c r="H8" s="1">
-        <v>2835</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -2296,7 +2296,7 @@
         <v>22</v>
       </c>
       <c r="H9" s="1">
-        <v>2827</v>
+        <v>2829</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -2322,7 +2322,7 @@
         <v>28</v>
       </c>
       <c r="H10" s="1">
-        <v>2051</v>
+        <v>2044</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -2345,7 +2345,7 @@
         <v>29</v>
       </c>
       <c r="H11" s="1">
-        <v>2027</v>
+        <v>2008</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -2368,7 +2368,7 @@
         <v>35</v>
       </c>
       <c r="H12" s="1">
-        <v>1988</v>
+        <v>1976</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -2394,7 +2394,7 @@
         <v>39</v>
       </c>
       <c r="H13" s="1">
-        <v>1601</v>
+        <v>1591</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -2417,7 +2417,7 @@
         <v>41</v>
       </c>
       <c r="H14" s="1">
-        <v>1453</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
@@ -2440,7 +2440,7 @@
         <v>42</v>
       </c>
       <c r="H15" s="1">
-        <v>1371</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
@@ -2448,9 +2448,12 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>45</v>
       </c>
       <c r="E16" s="1" t="s">
@@ -2463,7 +2466,7 @@
         <v>45</v>
       </c>
       <c r="H16" s="1">
-        <v>1329</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
@@ -2471,12 +2474,9 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="1" t="s">
         <v>48</v>
       </c>
       <c r="E17" s="1" t="s">
@@ -2489,7 +2489,7 @@
         <v>48</v>
       </c>
       <c r="H17" s="1">
-        <v>1328</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -2515,7 +2515,7 @@
         <v>54</v>
       </c>
       <c r="H18" s="1">
-        <v>1259</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
@@ -2538,7 +2538,7 @@
         <v>57</v>
       </c>
       <c r="H19" s="1">
-        <v>1239</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
@@ -2561,7 +2561,7 @@
         <v>59</v>
       </c>
       <c r="H20" s="1">
-        <v>1147</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
@@ -2584,7 +2584,7 @@
         <v>60</v>
       </c>
       <c r="H21" s="1">
-        <v>1122</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
@@ -2633,7 +2633,7 @@
         <v>68</v>
       </c>
       <c r="H23" s="1">
-        <v>1039</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
@@ -2656,7 +2656,7 @@
         <v>70</v>
       </c>
       <c r="H24" s="1">
-        <v>1032</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
@@ -2679,7 +2679,7 @@
         <v>72</v>
       </c>
       <c r="H25" s="1">
-        <v>1031</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -2702,7 +2702,7 @@
         <v>74</v>
       </c>
       <c r="H26" s="1">
-        <v>982</v>
+        <v>993</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -2725,7 +2725,7 @@
         <v>76</v>
       </c>
       <c r="H27" s="1">
-        <v>970</v>
+        <v>962</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -2748,7 +2748,7 @@
         <v>79</v>
       </c>
       <c r="H28" s="1">
-        <v>964</v>
+        <v>959</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
@@ -2759,10 +2759,10 @@
         <v>0</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>80</v>
@@ -2771,7 +2771,7 @@
         <v>81</v>
       </c>
       <c r="H29" s="1">
-        <v>939</v>
+        <v>935</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
@@ -2779,22 +2779,22 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="G30" s="1" t="s">
-        <v>84</v>
-      </c>
       <c r="H30" s="1">
-        <v>936</v>
+        <v>932</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
@@ -2802,13 +2802,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>85</v>
@@ -2817,7 +2817,7 @@
         <v>86</v>
       </c>
       <c r="H31" s="1">
-        <v>924</v>
+        <v>927</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
@@ -2828,7 +2828,7 @@
         <v>7</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>87</v>
@@ -2843,7 +2843,7 @@
         <v>87</v>
       </c>
       <c r="H32" s="1">
-        <v>880</v>
+        <v>867</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
@@ -2889,7 +2889,7 @@
         <v>93</v>
       </c>
       <c r="H34" s="1">
-        <v>818</v>
+        <v>816</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
@@ -2912,7 +2912,7 @@
         <v>95</v>
       </c>
       <c r="H35" s="1">
-        <v>799</v>
+        <v>803</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
@@ -2920,13 +2920,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>96</v>
@@ -2935,7 +2935,7 @@
         <v>97</v>
       </c>
       <c r="H36" s="1">
-        <v>798</v>
+        <v>797</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
@@ -2943,13 +2943,13 @@
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>98</v>
@@ -2969,10 +2969,10 @@
         <v>7</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>100</v>
@@ -2981,7 +2981,7 @@
         <v>101</v>
       </c>
       <c r="H38" s="1">
-        <v>744</v>
+        <v>746</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
@@ -3004,7 +3004,7 @@
         <v>103</v>
       </c>
       <c r="H39" s="1">
-        <v>737</v>
+        <v>732</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
@@ -3030,7 +3030,7 @@
         <v>105</v>
       </c>
       <c r="H40" s="1">
-        <v>698</v>
+        <v>695</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
@@ -3044,10 +3044,10 @@
         <v>13</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>106</v>
@@ -3056,7 +3056,7 @@
         <v>107</v>
       </c>
       <c r="H41" s="1">
-        <v>696</v>
+        <v>690</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
@@ -3067,10 +3067,10 @@
         <v>0</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>108</v>
@@ -3079,7 +3079,7 @@
         <v>109</v>
       </c>
       <c r="H42" s="1">
-        <v>675</v>
+        <v>688</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -3087,13 +3087,16 @@
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>16</v>
+        <v>48</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>87</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>17</v>
+        <v>88</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>110</v>
@@ -3125,7 +3128,7 @@
         <v>113</v>
       </c>
       <c r="H44" s="1">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
@@ -3133,16 +3136,13 @@
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>87</v>
+        <v>4</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>88</v>
+        <v>5</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>114</v>
@@ -3151,7 +3151,7 @@
         <v>115</v>
       </c>
       <c r="H45" s="1">
-        <v>673</v>
+        <v>667</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
@@ -3174,7 +3174,7 @@
         <v>117</v>
       </c>
       <c r="H46" s="1">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
@@ -3185,10 +3185,10 @@
         <v>0</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>118</v>
@@ -3197,7 +3197,7 @@
         <v>119</v>
       </c>
       <c r="H47" s="1">
-        <v>655</v>
+        <v>653</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
@@ -3208,10 +3208,10 @@
         <v>0</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>120</v>
@@ -3220,7 +3220,7 @@
         <v>121</v>
       </c>
       <c r="H48" s="1">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
@@ -3231,10 +3231,10 @@
         <v>0</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>122</v>
@@ -3243,7 +3243,7 @@
         <v>123</v>
       </c>
       <c r="H49" s="1">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
@@ -3266,7 +3266,7 @@
         <v>107</v>
       </c>
       <c r="H50" s="1">
-        <v>633</v>
+        <v>627</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
@@ -3289,7 +3289,7 @@
         <v>126</v>
       </c>
       <c r="H51" s="1">
-        <v>628</v>
+        <v>620</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
@@ -3297,13 +3297,13 @@
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>127</v>
@@ -3312,7 +3312,7 @@
         <v>128</v>
       </c>
       <c r="H52" s="1">
-        <v>614</v>
+        <v>619</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
@@ -3323,10 +3323,10 @@
         <v>0</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>129</v>
@@ -3358,7 +3358,7 @@
         <v>132</v>
       </c>
       <c r="H54" s="1">
-        <v>612</v>
+        <v>610</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
@@ -3369,13 +3369,10 @@
         <v>7</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>52</v>
+        <v>11</v>
       </c>
       <c r="F55" s="1" t="s">
         <v>133</v>
@@ -3384,7 +3381,7 @@
         <v>134</v>
       </c>
       <c r="H55" s="1">
-        <v>604</v>
+        <v>607</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
@@ -3392,13 +3389,13 @@
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>135</v>
@@ -3418,10 +3415,13 @@
         <v>7</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>51</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>137</v>
@@ -3430,7 +3430,7 @@
         <v>138</v>
       </c>
       <c r="H57" s="1">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
@@ -3453,7 +3453,7 @@
         <v>140</v>
       </c>
       <c r="H58" s="1">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
@@ -3476,7 +3476,7 @@
         <v>142</v>
       </c>
       <c r="H59" s="1">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
@@ -3487,10 +3487,10 @@
         <v>0</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>143</v>
@@ -3499,7 +3499,7 @@
         <v>144</v>
       </c>
       <c r="H60" s="1">
-        <v>577</v>
+        <v>571</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
@@ -3510,10 +3510,10 @@
         <v>0</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>145</v>
@@ -3522,7 +3522,7 @@
         <v>146</v>
       </c>
       <c r="H61" s="1">
-        <v>575</v>
+        <v>570</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.2">
@@ -3545,7 +3545,7 @@
         <v>148</v>
       </c>
       <c r="H62" s="1">
-        <v>570</v>
+        <v>567</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
@@ -3553,13 +3553,13 @@
         <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>149</v>
@@ -3568,7 +3568,7 @@
         <v>150</v>
       </c>
       <c r="H63" s="1">
-        <v>553</v>
+        <v>558</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
@@ -3576,13 +3576,13 @@
         <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="F64" s="1" t="s">
         <v>151</v>
@@ -3602,10 +3602,13 @@
         <v>0</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>42</v>
+        <v>60</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>63</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>153</v>
@@ -3614,7 +3617,7 @@
         <v>154</v>
       </c>
       <c r="H65" s="1">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
@@ -3625,13 +3628,10 @@
         <v>0</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>63</v>
+        <v>4</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>64</v>
+        <v>5</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>155</v>
@@ -3640,7 +3640,7 @@
         <v>156</v>
       </c>
       <c r="H66" s="1">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
@@ -3651,10 +3651,10 @@
         <v>0</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>157</v>
@@ -3663,7 +3663,7 @@
         <v>158</v>
       </c>
       <c r="H67" s="1">
-        <v>546</v>
+        <v>549</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
@@ -3674,10 +3674,10 @@
         <v>7</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F68" s="1" t="s">
         <v>159</v>
@@ -3686,7 +3686,7 @@
         <v>160</v>
       </c>
       <c r="H68" s="1">
-        <v>546</v>
+        <v>544</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
@@ -3709,7 +3709,7 @@
         <v>162</v>
       </c>
       <c r="H69" s="1">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
@@ -3720,10 +3720,13 @@
         <v>7</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="F70" s="1" t="s">
         <v>163</v>
@@ -3732,7 +3735,7 @@
         <v>164</v>
       </c>
       <c r="H70" s="1">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
@@ -3778,7 +3781,7 @@
         <v>168</v>
       </c>
       <c r="H72" s="1">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
@@ -3814,11 +3817,8 @@
       <c r="C74" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D74" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="E74" s="1" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>171</v>
@@ -3827,7 +3827,7 @@
         <v>172</v>
       </c>
       <c r="H74" s="1">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
@@ -3850,7 +3850,7 @@
         <v>174</v>
       </c>
       <c r="H75" s="1">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
@@ -3873,7 +3873,7 @@
         <v>176</v>
       </c>
       <c r="H76" s="1">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
@@ -3896,7 +3896,7 @@
         <v>178</v>
       </c>
       <c r="H77" s="1">
-        <v>511</v>
+        <v>507</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
@@ -3942,7 +3942,7 @@
         <v>182</v>
       </c>
       <c r="H79" s="1">
-        <v>475</v>
+        <v>484</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
@@ -3950,13 +3950,13 @@
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="F80" s="1" t="s">
         <v>183</v>
@@ -3965,7 +3965,7 @@
         <v>184</v>
       </c>
       <c r="H80" s="1">
-        <v>470</v>
+        <v>474</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.2">
@@ -3973,13 +3973,13 @@
         <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="F81" s="1" t="s">
         <v>185</v>
@@ -3988,7 +3988,7 @@
         <v>186</v>
       </c>
       <c r="H81" s="1">
-        <v>460</v>
+        <v>467</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.2">
@@ -4014,7 +4014,7 @@
         <v>188</v>
       </c>
       <c r="H82" s="1">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.2">
@@ -4048,7 +4048,7 @@
         <v>7</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D84" s="1" t="s">
         <v>87</v>
@@ -4063,7 +4063,7 @@
         <v>192</v>
       </c>
       <c r="H84" s="1">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
@@ -4071,13 +4071,13 @@
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F85" s="1" t="s">
         <v>193</v>
@@ -4086,7 +4086,7 @@
         <v>194</v>
       </c>
       <c r="H85" s="1">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.2">
@@ -4109,7 +4109,7 @@
         <v>196</v>
       </c>
       <c r="H86" s="1">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.2">
@@ -4117,13 +4117,13 @@
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>197</v>
@@ -4132,7 +4132,7 @@
         <v>198</v>
       </c>
       <c r="H87" s="1">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.2">
@@ -4155,7 +4155,7 @@
         <v>200</v>
       </c>
       <c r="H88" s="1">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.2">
@@ -4181,7 +4181,7 @@
         <v>202</v>
       </c>
       <c r="H89" s="1">
-        <v>413</v>
+        <v>417</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.2">
@@ -4204,7 +4204,7 @@
         <v>204</v>
       </c>
       <c r="H90" s="1">
-        <v>407</v>
+        <v>411</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.2">
@@ -4212,13 +4212,16 @@
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>4</v>
+        <v>7</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="F91" s="1" t="s">
         <v>205</v>
@@ -4235,16 +4238,13 @@
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D92" s="1" t="s">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="F92" s="1" t="s">
         <v>207</v>
@@ -4253,7 +4253,7 @@
         <v>208</v>
       </c>
       <c r="H92" s="1">
-        <v>401</v>
+        <v>407</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.2">
@@ -4276,7 +4276,7 @@
         <v>210</v>
       </c>
       <c r="H93" s="1">
-        <v>401</v>
+        <v>405</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.2">
@@ -4299,7 +4299,7 @@
         <v>212</v>
       </c>
       <c r="H94" s="1">
-        <v>395</v>
+        <v>401</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.2">
@@ -4322,7 +4322,7 @@
         <v>214</v>
       </c>
       <c r="H95" s="1">
-        <v>394</v>
+        <v>398</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.2">
@@ -4333,10 +4333,10 @@
         <v>0</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="F96" s="1" t="s">
         <v>215</v>
@@ -4345,7 +4345,7 @@
         <v>216</v>
       </c>
       <c r="H96" s="1">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.2">
@@ -4356,10 +4356,10 @@
         <v>0</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>17</v>
+        <v>61</v>
       </c>
       <c r="F97" s="1" t="s">
         <v>217</v>
@@ -4368,7 +4368,7 @@
         <v>218</v>
       </c>
       <c r="H97" s="1">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.2">
@@ -4376,16 +4376,13 @@
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D98" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F98" s="1" t="s">
         <v>219</v>
@@ -4394,7 +4391,7 @@
         <v>220</v>
       </c>
       <c r="H98" s="1">
-        <v>383</v>
+        <v>389</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.2">
@@ -4405,10 +4402,10 @@
         <v>0</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="F99" s="1" t="s">
         <v>221</v>
@@ -4417,7 +4414,7 @@
         <v>222</v>
       </c>
       <c r="H99" s="1">
-        <v>383</v>
+        <v>386</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.2">
@@ -4425,13 +4422,13 @@
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="F100" s="1" t="s">
         <v>223</v>
@@ -4440,7 +4437,7 @@
         <v>224</v>
       </c>
       <c r="H100" s="1">
-        <v>374</v>
+        <v>382</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.2">
@@ -4448,13 +4445,16 @@
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F101" s="1" t="s">
         <v>225</v>
@@ -4463,7 +4463,7 @@
         <v>226</v>
       </c>
       <c r="H101" s="1">
-        <v>370</v>
+        <v>379</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.2">
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="F102" s="1" t="s">
         <v>227</v>
@@ -4486,7 +4486,7 @@
         <v>228</v>
       </c>
       <c r="H102" s="1">
-        <v>369</v>
+        <v>377</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.2">
@@ -4497,10 +4497,10 @@
         <v>7</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>82</v>
+        <v>8</v>
       </c>
       <c r="F103" s="1" t="s">
         <v>229</v>
@@ -4509,7 +4509,7 @@
         <v>230</v>
       </c>
       <c r="H103" s="1">
-        <v>368</v>
+        <v>375</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.2">
@@ -4532,7 +4532,7 @@
         <v>232</v>
       </c>
       <c r="H104" s="1">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.2">
@@ -4540,13 +4540,13 @@
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>233</v>
@@ -4555,7 +4555,7 @@
         <v>234</v>
       </c>
       <c r="H105" s="1">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.2">
@@ -4566,13 +4566,10 @@
         <v>0</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D106" s="1" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>235</v>
@@ -4592,10 +4589,13 @@
         <v>0</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>60</v>
+        <v>13</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>45</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>237</v>
@@ -4604,7 +4604,7 @@
         <v>238</v>
       </c>
       <c r="H107" s="1">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.2">
@@ -4615,10 +4615,10 @@
         <v>0</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>239</v>
@@ -4627,7 +4627,7 @@
         <v>240</v>
       </c>
       <c r="H108" s="1">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.2">
@@ -4638,13 +4638,10 @@
         <v>0</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D109" s="1" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="F109" s="1" t="s">
         <v>241</v>
@@ -4666,8 +4663,11 @@
       <c r="C110" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="D110" s="1" t="s">
+        <v>45</v>
+      </c>
       <c r="E110" s="1" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="F110" s="1" t="s">
         <v>243</v>
@@ -4676,7 +4676,7 @@
         <v>244</v>
       </c>
       <c r="H110" s="1">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.2">
@@ -4722,7 +4722,7 @@
         <v>248</v>
       </c>
       <c r="H112" s="1">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.2">
@@ -4730,13 +4730,13 @@
         <v>112</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>249</v>
@@ -4745,7 +4745,7 @@
         <v>250</v>
       </c>
       <c r="H113" s="1">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.2">
@@ -4768,7 +4768,7 @@
         <v>252</v>
       </c>
       <c r="H114" s="1">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.2">
@@ -4779,10 +4779,10 @@
         <v>0</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>253</v>
@@ -4791,7 +4791,7 @@
         <v>254</v>
       </c>
       <c r="H115" s="1">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.2">
@@ -4814,7 +4814,7 @@
         <v>256</v>
       </c>
       <c r="H116" s="1">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.2">
@@ -4822,13 +4822,13 @@
         <v>116</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="F117" s="1" t="s">
         <v>257</v>
@@ -4837,7 +4837,7 @@
         <v>258</v>
       </c>
       <c r="H117" s="1">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.2">
@@ -4860,7 +4860,7 @@
         <v>260</v>
       </c>
       <c r="H118" s="1">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.2">
@@ -4871,13 +4871,10 @@
         <v>7</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D119" s="1" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="F119" s="1" t="s">
         <v>261</v>
@@ -4886,7 +4883,7 @@
         <v>262</v>
       </c>
       <c r="H119" s="1">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.2">
@@ -4894,13 +4891,13 @@
         <v>119</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="F120" s="1" t="s">
         <v>263</v>
@@ -4909,7 +4906,7 @@
         <v>264</v>
       </c>
       <c r="H120" s="1">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.2">
@@ -4917,13 +4914,16 @@
         <v>120</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>60</v>
+        <v>7</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="F121" s="1" t="s">
         <v>265</v>
@@ -4932,7 +4932,7 @@
         <v>266</v>
       </c>
       <c r="H121" s="1">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.2">
@@ -4940,19 +4940,19 @@
         <v>121</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>267</v>
       </c>
       <c r="G122" s="1" t="s">
-        <v>162</v>
+        <v>268</v>
       </c>
       <c r="H122" s="1">
         <v>335</v>
@@ -4963,22 +4963,22 @@
         <v>122</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E123" s="1" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F123" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G123" s="1" t="s">
-        <v>269</v>
+        <v>172</v>
       </c>
       <c r="H123" s="1">
-        <v>330</v>
+        <v>335</v>
       </c>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.2">
@@ -5001,7 +5001,7 @@
         <v>271</v>
       </c>
       <c r="H124" s="1">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.2">
@@ -5009,13 +5009,13 @@
         <v>124</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="E125" s="1" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F125" s="1" t="s">
         <v>272</v>
@@ -5024,7 +5024,7 @@
         <v>273</v>
       </c>
       <c r="H125" s="1">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.2">
@@ -5055,13 +5055,13 @@
         <v>126</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="E127" s="1" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="F127" s="1" t="s">
         <v>276</v>
@@ -5070,7 +5070,7 @@
         <v>277</v>
       </c>
       <c r="H127" s="1">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.2">
@@ -5096,7 +5096,7 @@
         <v>279</v>
       </c>
       <c r="H128" s="1">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.2">
@@ -5107,10 +5107,10 @@
         <v>0</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="E129" s="1" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="F129" s="1" t="s">
         <v>280</v>
@@ -5119,7 +5119,7 @@
         <v>281</v>
       </c>
       <c r="H129" s="1">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.2">
@@ -5130,10 +5130,10 @@
         <v>0</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E130" s="1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F130" s="1" t="s">
         <v>282</v>
@@ -5165,7 +5165,7 @@
         <v>285</v>
       </c>
       <c r="H131" s="1">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.2">
@@ -5176,10 +5176,10 @@
         <v>0</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="E132" s="1" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F132" s="1" t="s">
         <v>286</v>
@@ -5188,7 +5188,7 @@
         <v>287</v>
       </c>
       <c r="H132" s="1">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.2">
@@ -5202,10 +5202,10 @@
         <v>13</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E133" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F133" s="1" t="s">
         <v>288</v>
@@ -5214,7 +5214,7 @@
         <v>289</v>
       </c>
       <c r="H133" s="1">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.2">
@@ -5237,7 +5237,7 @@
         <v>291</v>
       </c>
       <c r="H134" s="1">
-        <v>297</v>
+        <v>294</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.2">
@@ -5283,7 +5283,7 @@
         <v>295</v>
       </c>
       <c r="H136" s="1">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.2">
@@ -5306,7 +5306,7 @@
         <v>297</v>
       </c>
       <c r="H137" s="1">
-        <v>289</v>
+        <v>281</v>
       </c>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.2">
@@ -5314,13 +5314,13 @@
         <v>137</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E138" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F138" s="1" t="s">
         <v>298</v>
@@ -5329,7 +5329,7 @@
         <v>299</v>
       </c>
       <c r="H138" s="1">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.2">
@@ -5352,7 +5352,7 @@
         <v>301</v>
       </c>
       <c r="H139" s="1">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.2">
@@ -5375,7 +5375,7 @@
         <v>303</v>
       </c>
       <c r="H140" s="1">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.2">
@@ -5383,16 +5383,13 @@
         <v>140</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D141" s="1" t="s">
-        <v>63</v>
+        <v>7</v>
       </c>
       <c r="E141" s="1" t="s">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="F141" s="1" t="s">
         <v>304</v>
@@ -5401,7 +5398,7 @@
         <v>305</v>
       </c>
       <c r="H141" s="1">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="142" spans="1:8" x14ac:dyDescent="0.2">
@@ -5412,10 +5409,13 @@
         <v>0</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>4</v>
+        <v>60</v>
+      </c>
+      <c r="D142" s="1" t="s">
+        <v>63</v>
       </c>
       <c r="E142" s="1" t="s">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="F142" s="1" t="s">
         <v>306</v>
@@ -5424,7 +5424,7 @@
         <v>307</v>
       </c>
       <c r="H142" s="1">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.2">
@@ -5432,16 +5432,13 @@
         <v>142</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D143" s="1" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="E143" s="1" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="F143" s="1" t="s">
         <v>308</v>
@@ -5450,7 +5447,7 @@
         <v>309</v>
       </c>
       <c r="H143" s="1">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.2">
@@ -5458,13 +5455,16 @@
         <v>143</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>22</v>
+        <v>7</v>
+      </c>
+      <c r="D144" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="E144" s="1" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="F144" s="1" t="s">
         <v>310</v>
@@ -5473,7 +5473,7 @@
         <v>311</v>
       </c>
       <c r="H144" s="1">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.2">
@@ -5484,10 +5484,10 @@
         <v>0</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E145" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F145" s="1" t="s">
         <v>312</v>
@@ -5496,7 +5496,7 @@
         <v>313</v>
       </c>
       <c r="H145" s="1">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.2">
@@ -5519,7 +5519,7 @@
         <v>315</v>
       </c>
       <c r="H146" s="1">
-        <v>269</v>
+        <v>264</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.2">
@@ -5530,10 +5530,10 @@
         <v>0</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="E147" s="1" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="F147" s="1" t="s">
         <v>316</v>
@@ -5542,7 +5542,7 @@
         <v>317</v>
       </c>
       <c r="H147" s="1">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.2">
@@ -5553,10 +5553,10 @@
         <v>0</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E148" s="1" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="F148" s="1" t="s">
         <v>318</v>
@@ -5565,7 +5565,7 @@
         <v>319</v>
       </c>
       <c r="H148" s="1">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.2">
@@ -5576,10 +5576,13 @@
         <v>0</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>32</v>
+        <v>60</v>
+      </c>
+      <c r="D149" s="1" t="s">
+        <v>63</v>
       </c>
       <c r="E149" s="1" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="F149" s="1" t="s">
         <v>320</v>
@@ -5588,7 +5591,7 @@
         <v>321</v>
       </c>
       <c r="H149" s="1">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.2">
@@ -5596,13 +5599,13 @@
         <v>149</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="E150" s="1" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="F150" s="1" t="s">
         <v>322</v>
@@ -5622,10 +5625,10 @@
         <v>0</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E151" s="1" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F151" s="1" t="s">
         <v>324</v>
@@ -5634,7 +5637,7 @@
         <v>325</v>
       </c>
       <c r="H151" s="1">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.2">
@@ -5645,10 +5648,10 @@
         <v>7</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E152" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F152" s="1" t="s">
         <v>326</v>
@@ -5657,7 +5660,7 @@
         <v>327</v>
       </c>
       <c r="H152" s="1">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.2">
@@ -5665,13 +5668,13 @@
         <v>152</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E153" s="1" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F153" s="1" t="s">
         <v>328</v>
@@ -5680,7 +5683,7 @@
         <v>329</v>
       </c>
       <c r="H153" s="1">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.2">
@@ -5691,13 +5694,10 @@
         <v>0</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D154" s="1" t="s">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="E154" s="1" t="s">
-        <v>64</v>
+        <v>23</v>
       </c>
       <c r="F154" s="1" t="s">
         <v>330</v>
@@ -5706,7 +5706,7 @@
         <v>331</v>
       </c>
       <c r="H154" s="1">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.2">
@@ -5717,10 +5717,13 @@
         <v>0</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>22</v>
+        <v>60</v>
+      </c>
+      <c r="D155" s="1" t="s">
+        <v>63</v>
       </c>
       <c r="E155" s="1" t="s">
-        <v>23</v>
+        <v>64</v>
       </c>
       <c r="F155" s="1" t="s">
         <v>332</v>
@@ -5729,7 +5732,7 @@
         <v>333</v>
       </c>
       <c r="H155" s="1">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.2">
@@ -5752,7 +5755,7 @@
         <v>335</v>
       </c>
       <c r="H156" s="1">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.2">
@@ -5763,10 +5766,10 @@
         <v>0</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E157" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F157" s="1" t="s">
         <v>336</v>
@@ -5775,7 +5778,7 @@
         <v>337</v>
       </c>
       <c r="H157" s="1">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.2">
@@ -5786,13 +5789,10 @@
         <v>0</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D158" s="1" t="s">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="E158" s="1" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="F158" s="1" t="s">
         <v>338</v>
@@ -5801,7 +5801,7 @@
         <v>339</v>
       </c>
       <c r="H158" s="1">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.2">
@@ -5812,10 +5812,10 @@
         <v>0</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E159" s="1" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F159" s="1" t="s">
         <v>340</v>
@@ -5824,7 +5824,7 @@
         <v>341</v>
       </c>
       <c r="H159" s="1">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.2">
@@ -5844,10 +5844,10 @@
         <v>342</v>
       </c>
       <c r="G160" s="1" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H160" s="1">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.2">
@@ -5881,19 +5881,19 @@
         <v>7</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E162" s="1" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F162" s="1" t="s">
         <v>345</v>
       </c>
       <c r="G162" s="1" t="s">
-        <v>68</v>
+        <v>346</v>
       </c>
       <c r="H162" s="1">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.2">
@@ -5904,19 +5904,19 @@
         <v>7</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E163" s="1" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F163" s="1" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G163" s="1" t="s">
-        <v>347</v>
+        <v>68</v>
       </c>
       <c r="H163" s="1">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.2">
@@ -5924,13 +5924,13 @@
         <v>163</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="E164" s="1" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="F164" s="1" t="s">
         <v>348</v>
@@ -5939,7 +5939,7 @@
         <v>349</v>
       </c>
       <c r="H164" s="1">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.2">
@@ -5950,19 +5950,19 @@
         <v>7</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="E165" s="1" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F165" s="1" t="s">
         <v>350</v>
       </c>
       <c r="G165" s="1" t="s">
-        <v>4</v>
+        <v>351</v>
       </c>
       <c r="H165" s="1">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.2">
@@ -5970,22 +5970,22 @@
         <v>165</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C166" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E166" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F166" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="G166" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E166" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F166" s="1" t="s">
-        <v>351</v>
-      </c>
-      <c r="G166" s="1" t="s">
-        <v>352</v>
-      </c>
       <c r="H166" s="1">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.2">
@@ -5998,20 +5998,17 @@
       <c r="C167" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D167" s="1" t="s">
-        <v>51</v>
-      </c>
       <c r="E167" s="1" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="F167" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G167" s="1" t="s">
-        <v>68</v>
+        <v>354</v>
       </c>
       <c r="H167" s="1">
-        <v>219</v>
+        <v>223</v>
       </c>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.2">
@@ -6024,17 +6021,20 @@
       <c r="C168" s="1" t="s">
         <v>29</v>
       </c>
+      <c r="D168" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="E168" s="1" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="F168" s="1" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G168" s="1" t="s">
-        <v>355</v>
+        <v>68</v>
       </c>
       <c r="H168" s="1">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.2">
@@ -6042,13 +6042,13 @@
         <v>168</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="E169" s="1" t="s">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="F169" s="1" t="s">
         <v>356</v>
@@ -6057,7 +6057,7 @@
         <v>357</v>
       </c>
       <c r="H169" s="1">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.2">
@@ -6068,10 +6068,10 @@
         <v>7</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="E170" s="1" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F170" s="1" t="s">
         <v>358</v>
@@ -6080,7 +6080,7 @@
         <v>359</v>
       </c>
       <c r="H170" s="1">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.2">
@@ -6103,7 +6103,7 @@
         <v>361</v>
       </c>
       <c r="H171" s="1">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.2">
@@ -6126,7 +6126,7 @@
         <v>363</v>
       </c>
       <c r="H172" s="1">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="173" spans="1:8" x14ac:dyDescent="0.2">
@@ -6137,10 +6137,10 @@
         <v>7</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E173" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F173" s="1" t="s">
         <v>364</v>
@@ -6149,7 +6149,7 @@
         <v>365</v>
       </c>
       <c r="H173" s="1">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.2">
@@ -6157,13 +6157,13 @@
         <v>173</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E174" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F174" s="1" t="s">
         <v>366</v>
@@ -6172,7 +6172,7 @@
         <v>367</v>
       </c>
       <c r="H174" s="1">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.2">
@@ -6198,7 +6198,7 @@
         <v>369</v>
       </c>
       <c r="H175" s="1">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.2">
@@ -6221,7 +6221,7 @@
         <v>371</v>
       </c>
       <c r="H176" s="1">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="177" spans="1:8" x14ac:dyDescent="0.2">
@@ -6244,7 +6244,7 @@
         <v>373</v>
       </c>
       <c r="H177" s="1">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="178" spans="1:8" x14ac:dyDescent="0.2">
@@ -6255,10 +6255,10 @@
         <v>7</v>
       </c>
       <c r="C178" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E178" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F178" s="1" t="s">
         <v>374</v>
@@ -6267,7 +6267,7 @@
         <v>375</v>
       </c>
       <c r="H178" s="1">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="179" spans="1:8" x14ac:dyDescent="0.2">
@@ -6293,7 +6293,7 @@
         <v>377</v>
       </c>
       <c r="H179" s="1">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="180" spans="1:8" x14ac:dyDescent="0.2">
@@ -6316,7 +6316,7 @@
         <v>379</v>
       </c>
       <c r="H180" s="1">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="181" spans="1:8" x14ac:dyDescent="0.2">
@@ -6339,7 +6339,7 @@
         <v>381</v>
       </c>
       <c r="H181" s="1">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="182" spans="1:8" x14ac:dyDescent="0.2">
@@ -6362,7 +6362,7 @@
         <v>4</v>
       </c>
       <c r="H182" s="1">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="183" spans="1:8" x14ac:dyDescent="0.2">
@@ -6385,7 +6385,7 @@
         <v>384</v>
       </c>
       <c r="H183" s="1">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="184" spans="1:8" x14ac:dyDescent="0.2">
@@ -6408,7 +6408,7 @@
         <v>386</v>
       </c>
       <c r="H184" s="1">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="185" spans="1:8" x14ac:dyDescent="0.2">
@@ -6434,7 +6434,7 @@
         <v>388</v>
       </c>
       <c r="H185" s="1">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>